<commit_message>
adjust docs of phases
</commit_message>
<xml_diff>
--- a/Plan AI-Driven Resource Tuning.xlsx
+++ b/Plan AI-Driven Resource Tuning.xlsx
@@ -59,7 +59,7 @@
     <t>Spark execution internals: Application → Job → Stage → Task; Driver/Executor; Partition &amp; Parallelism; Executor Resource Model; Spark resource configuration; YARN architecture và resource allocation; Spark History Server, EventLog, YARN RM API</t>
   </si>
   <si>
-    <t>Xác minh LOCAL_YARN_V1; đo capacity thực tế; resolve config C1; tạo DATA_DEBUG_V1; chạy W03_JOIN_V1 với EXP_001; lấy spark_application_id; xây Spark History Server collector, YARN RM collector; lưu raw payload và metadata</t>
+    <t>Xác minh LOCAL_YARN_V1; đo capacity thực tế; hoàn tất các review gate TPC-DS; resolve config C1; materialize TPCDS_DEBUG version 1; chỉ sau phê duyệt mới chạy W03_TPCDS_JOIN version 1 với EXP_001; lấy spark_application_id; xây Spark History Server collector, YARN RM collector; lưu raw payload và metadata</t>
   </si>
   <si>
     <t>Spark-on-YARN benchmark chạy được; có ít nhất một execution trace được từ experiment → Spark/YARN raw evidence; hoàn thiện Data Gate</t>
@@ -83,7 +83,7 @@
     <t>Statistics cơ bản: mean, variance, std, percentile, outlier, correlation, noise; experimental design; đồng thời bắt đầu ML fundamentals: supervised learning, X/y, regression, train/validation/test, MAE/MAPE/RMSE/R²</t>
   </si>
   <si>
-    <t>Thiết kế và chạy systematic benchmark với các workload FILTER, AGGREGATION, JOIN, SHUFFLE_HEAVY, SKEW_JOIN; thử nhiều input scale và vùng resource under/reasonable/over-provisioned; repeat một số config; tạo dataset lịch sử. Song song train Pilot Model P0 để kiểm tra dataset/feature có đủ signal hay không</t>
+    <t>Thiết kế và chạy TPC-DS-based controlled benchmark với W01_TPCDS_SCAN, W02_TPCDS_AGG, W03_TPCDS_JOIN, W04_TPCDS_MULTI_JOIN, W05_TPCDS_SHUFFLE_SORT, W06_TPCDS_COMPLEX_SQL (workload_version 1); dùng TPCDS_DEBUG và TPCDS_SF1 (dataset_version 1); thử các vùng resource under/reasonable/over-provisioned; repeat một số config; profile coverage/skew từ dữ liệu quan sát; tạo dataset lịch sử. Song song train Pilot Model P0 để kiểm tra dataset/feature có đủ signal hay không</t>
   </si>
   <si>
     <t>Historical execution dataset có workload/config diversity; biết sparse region và measurement noise; có pilot runtime model đầu tiên nhưng chưa coi là model chính thức</t>

</xml_diff>